<commit_message>
Update Availability.xlsx with latest collector schedules
Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Availability.xlsx
+++ b/Availability.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/522f0e7f2c00dc23/Documents/College/Spring 2026/XXX_____Research/Claude Code Setup Data/Collector_Schedule/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/522f0e7f2c00dc23/Documents/College/Spring-2026/XXX_____Research/Claude Code Setup Data/Collector_Schedule/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="103" documentId="11_485854879254DF546F882B8A982F9F8FB616C25A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E6131F4F-A7DB-4612-A8B0-05E5F4BD6725}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1FC6104B-2FC8-4CE5-9389-C767F22EBFCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="2135" yWindow="2135" windowWidth="14400" windowHeight="7290" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="90" yWindow="315" windowWidth="29010" windowHeight="15240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SOT" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="11">
   <si>
     <t>Mon</t>
   </si>
@@ -61,6 +61,9 @@
   </si>
   <si>
     <t>PM</t>
+  </si>
+  <si>
+    <t>e</t>
   </si>
 </sst>
 </file>
@@ -436,13 +439,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:I5"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="6" customWidth="1"/>
     <col min="3" max="9" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
@@ -465,7 +468,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
@@ -489,7 +492,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>8</v>
       </c>
@@ -507,7 +510,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
@@ -535,13 +538,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="B2:I5"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="6" customWidth="1"/>
     <col min="3" max="9" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
@@ -564,7 +567,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
@@ -576,7 +579,7 @@
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>8</v>
       </c>
@@ -588,7 +591,7 @@
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
@@ -608,13 +611,13 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="B2:I5"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="6" customWidth="1"/>
     <col min="3" max="9" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
@@ -637,7 +640,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
@@ -649,7 +652,7 @@
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>8</v>
       </c>
@@ -661,7 +664,7 @@
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
@@ -681,13 +684,13 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="B2:I5"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="6" customWidth="1"/>
     <col min="3" max="9" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
@@ -710,7 +713,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
@@ -722,7 +725,7 @@
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>8</v>
       </c>
@@ -734,7 +737,7 @@
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
@@ -753,14 +756,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="B2:I5"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <dimension ref="A2:I5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="6" customWidth="1"/>
     <col min="3" max="9" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
@@ -783,7 +786,10 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
       <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
@@ -805,7 +811,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>8</v>
       </c>
@@ -825,7 +831,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
@@ -855,13 +861,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B2:I5"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="6" customWidth="1"/>
     <col min="3" max="9" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
@@ -884,7 +890,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
@@ -910,7 +916,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>8</v>
       </c>
@@ -930,7 +936,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
@@ -958,13 +964,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="B2:I5"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="6" customWidth="1"/>
     <col min="3" max="9" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
@@ -987,7 +993,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
@@ -1009,7 +1015,7 @@
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>8</v>
       </c>
@@ -1023,7 +1029,7 @@
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
@@ -1043,13 +1049,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB1992FA-6492-4E43-95C1-271D1F73EDEE}">
   <dimension ref="B2:I5"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="6" customWidth="1"/>
     <col min="3" max="9" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1072,7 +1078,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
@@ -1088,7 +1094,7 @@
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>8</v>
       </c>
@@ -1104,7 +1110,7 @@
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
@@ -1130,13 +1136,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="B2:I5"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="6" customWidth="1"/>
     <col min="3" max="9" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1159,7 +1165,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
@@ -1175,7 +1181,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>8</v>
       </c>
@@ -1191,7 +1197,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
@@ -1217,13 +1223,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="B2:I5"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="6" customWidth="1"/>
     <col min="3" max="9" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1246,7 +1252,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
@@ -1264,7 +1270,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>8</v>
       </c>
@@ -1280,7 +1286,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
@@ -1312,13 +1318,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="B2:I5"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="6" customWidth="1"/>
     <col min="3" max="9" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1341,7 +1347,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
@@ -1367,7 +1373,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>8</v>
       </c>
@@ -1375,13 +1381,15 @@
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
+      <c r="G4" s="2">
+        <v>1</v>
+      </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
@@ -1401,13 +1409,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="B2:I5"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="6" customWidth="1"/>
     <col min="3" max="9" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1430,7 +1438,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
@@ -1454,7 +1462,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>8</v>
       </c>
@@ -1470,7 +1478,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.75">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
@@ -1480,7 +1488,9 @@
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
+      <c r="G5" s="2">
+        <v>1</v>
+      </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2">
         <v>1</v>

</xml_diff>

<commit_message>
Update availability data and rebuild dashboard
Committed new Availability.xlsx from desktop and rebuilt
availability_heatmap.html and dashboard.html to reflect
updated collector schedule data.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Availability.xlsx
+++ b/Availability.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/522f0e7f2c00dc23/Documents/College/Spring-2026/XXX_____Research/Claude Code Setup Data/Collector_Schedule/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/522f0e7f2c00dc23/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{1FC6104B-2FC8-4CE5-9389-C767F22EBFCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{916800B3-66B4-4DB8-A9FC-27183F5C58E9}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DE9094AB-3F78-4A68-AF01-4BA2F98E2DE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="90" yWindow="315" windowWidth="29010" windowHeight="15240" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SOT" sheetId="1" r:id="rId1"/>
@@ -22,16 +22,13 @@
     <sheet name="JEN" sheetId="6" r:id="rId7"/>
     <sheet name="SCT" sheetId="7" r:id="rId8"/>
     <sheet name="TER" sheetId="8" r:id="rId9"/>
-    <sheet name="PRA" sheetId="9" r:id="rId10"/>
-    <sheet name="NAT" sheetId="10" r:id="rId11"/>
-    <sheet name="NRS" sheetId="11" r:id="rId12"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="11">
   <si>
     <t>Mon</t>
   </si>
@@ -535,225 +532,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="B2:I5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="6" customWidth="1"/>
-    <col min="3" max="9" width="10" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-    </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-    </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="B2:I5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="6" customWidth="1"/>
-    <col min="3" max="9" width="10" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-    </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-    </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="B2:I5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="6" customWidth="1"/>
-    <col min="3" max="9" width="10" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-    </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-    </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A2:I5"/>
@@ -816,7 +594,9 @@
         <v>8</v>
       </c>
       <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
+      <c r="D4" s="2">
+        <v>1</v>
+      </c>
       <c r="E4" s="2"/>
       <c r="F4" s="2">
         <v>1</v>
@@ -839,7 +619,9 @@
         <v>1</v>
       </c>
       <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
+      <c r="E5" s="2">
+        <v>1</v>
+      </c>
       <c r="F5" s="2">
         <v>1</v>
       </c>
@@ -1398,7 +1180,9 @@
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
+      <c r="F5" s="2">
+        <v>1</v>
+      </c>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>

</xml_diff>